<commit_message>
Add automation demo and updated outputs
</commit_message>
<xml_diff>
--- a/daily_report_2026-09-30.xlsx
+++ b/daily_report_2026-09-30.xlsx
@@ -483,12 +483,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>16:01:10</t>
+          <t>16:48:40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>32°C</t>
+          <t>31°C</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>77%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>